<commit_message>
Publication build from 1b6bbe0d88ab3535fdebc34d4134d4104e73b7b9 (v0.1.0)
</commit_message>
<xml_diff>
--- a/publication/web-root/matchsync-donor/0.1.0/CodeSystem-nmdp-donor-status.xlsx
+++ b/publication/web-root/matchsync-donor/0.1.0/CodeSystem-nmdp-donor-status.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
   <si>
     <t>Property</t>
   </si>
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://terminology.nmdp.org/codesystem/donor-status</t>
+    <t>http://fhir.nmdp.org/CodeSystem/donor-status</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-02T19:29:11+00:00</t>
+    <t>2026-09-03T14:51:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,8 @@
     <t>Status codes for NMDP registered donors. These codes represent the
 enterprise Registry Status maintained by NMDP, indicating a donor's availability
 for patient search, matching, and product request activities. Source: ODS
-DonorWithSampleResponse (v05).</t>
+DonorWithSampleResponse (v05). In FHIR Donor API payloads, donor status is
+conveyed as a valueString on the donor-status extension.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -96,7 +97,7 @@
     <t>Case Sensitive</t>
   </si>
   <si>
-    <t>true</t>
+    <t>false</t>
   </si>
   <si>
     <t>Value Set (all codes)</t>
@@ -141,16 +142,13 @@
     <t>1</t>
   </si>
   <si>
-    <t>available</t>
-  </si>
-  <si>
     <t>Available</t>
   </si>
   <si>
     <t>Donor is available for search, further typing, and collection/transplant (ODS code: AV).</t>
   </si>
   <si>
-    <t>temporarily-unavailable</t>
+    <t>Temporarily-Unavailable</t>
   </si>
   <si>
     <t>Temporarily Unavailable</t>
@@ -159,16 +157,13 @@
     <t>Donor is temporarily unavailable, typically post-collection with a future available date (ODS code: TU).</t>
   </si>
   <si>
-    <t>active</t>
-  </si>
-  <si>
     <t>Active</t>
   </si>
   <si>
     <t>Donor is currently active on a search — reserved for a specific patient case (ODS code: AC).</t>
   </si>
   <si>
-    <t>permanently-unavailable</t>
+    <t>Permanently-Unavailable</t>
   </si>
   <si>
     <t>Permanently Unavailable</t>
@@ -507,10 +502,10 @@
         <v>41</v>
       </c>
       <c r="C2" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s" s="2">
         <v>42</v>
-      </c>
-      <c r="D2" t="s" s="2">
-        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -518,13 +513,13 @@
         <v>40</v>
       </c>
       <c r="B3" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="C3" t="s" s="2">
+      <c r="D3" t="s" s="2">
         <v>45</v>
-      </c>
-      <c r="D3" t="s" s="2">
-        <v>46</v>
       </c>
     </row>
     <row r="4">
@@ -532,13 +527,13 @@
         <v>40</v>
       </c>
       <c r="B4" t="s" s="2">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s" s="2">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s" s="2">
         <v>47</v>
-      </c>
-      <c r="C4" t="s" s="2">
-        <v>48</v>
-      </c>
-      <c r="D4" t="s" s="2">
-        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -546,13 +541,13 @@
         <v>40</v>
       </c>
       <c r="B5" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="D5" t="s" s="2">
         <v>50</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>51</v>
-      </c>
-      <c r="D5" t="s" s="2">
-        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>